<commit_message>
Unify reproductive cycles and correct lamb review scope
</commit_message>
<xml_diff>
--- a/web/public/downloads/eSheepPlus_全功能录入模板_v7.xlsx
+++ b/web/public/downloads/eSheepPlus_全功能录入模板_v7.xlsx
@@ -163,113 +163,125 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">产羔胎次</t>
+          <t xml:space="preserve">繁殖关联</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">产羔表不手填胎次，系统以产羔时间点之前的有效胎次自动加 1。</t>
+          <t xml:space="preserve">配种轮次填写新一轮配种或本轮补配；补配须填写关联配种记录ID或配种导入键。批量行按每只母羊分别关联；旧模板缺少关联时，仅在归属唯一明确时推导。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">羔羊称重</t>
+          <t xml:space="preserve">产羔胎次</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">填写体重时必须填写实际称重日期；出生 24 小时内记为初生重，超过 24 小时记为普通称重。未称重可同时留空。</t>
+          <t xml:space="preserve">产羔表不手填胎次，系统以产羔时间点之前的有效胎次自动加 1。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">断奶日增重</t>
+          <t xml:space="preserve">羔羊称重</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">系统以出生后、断奶前最早一条实际称重为起点自动计算；断奶表不填写初生重和日增重。没有有效称重时不计算。</t>
+          <t xml:space="preserve">填写体重时必须填写实际称重日期；出生 24 小时内记为初生重，超过 24 小时记为普通称重。未称重可同时留空。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">断奶调舍</t>
+          <t xml:space="preserve">断奶日增重</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">断奶不填写母本或胎只数；每条断奶必须填写转入圈舍，断奶事实与调舍在同一事务中提交。</t>
+          <t xml:space="preserve">系统以出生后、断奶前最早一条实际称重为起点自动计算；断奶表不填写初生重和日增重。没有有效称重时不计算。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">引用核对</t>
+          <t xml:space="preserve">断奶调舍</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">称重、断奶、转群等事件的耳号，以及圈舍、目录、库存批号、冻精等引用，必须已在当前牧场存在或在本文件前置工作表中创建。</t>
+          <t xml:space="preserve">断奶不填写母本或胎只数；每条断奶必须填写转入圈舍，断奶事实与调舍在同一事务中提交。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">批量列表</t>
+          <t xml:space="preserve">引用核对</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">多个耳号使用英文分号 ; 分隔。组合明细使用 | 分列、使用 ; 分条。</t>
+          <t xml:space="preserve">称重、断奶、转群等事件的耳号，以及圈舍、目录、库存批号、冻精等引用，必须已在当前牧场存在或在本文件前置工作表中创建。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">离场批次</t>
+          <t xml:space="preserve">批量列表</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">离场表每行代表同一次离场；可填写多个耳号。出售时只填写整批总售卖金额，不填写或推算单羊价格。</t>
+          <t xml:space="preserve">多个耳号使用英文分号 ; 分隔。组合明细使用 | 分列、使用 ; 分条。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">事务</t>
+          <t xml:space="preserve">离场批次</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">整份文件通过权限、业务校验、SwiftData、审计和 Outbox 管道一次提交；任一阻断错误会整批回滚。</t>
+          <t xml:space="preserve">离场表每行代表同一次离场；可填写多个耳号。出售时只填写整批总售卖金额，不填写或推算单羊价格。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t xml:space="preserve">事务</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">整份文件通过权限、业务校验、SwiftData、审计和 Outbox 管道一次提交；任一阻断错误会整批回滚。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t xml:space="preserve">不支持</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t xml:space="preserve">历史修正、撤销、恢复、删除不通过 Excel 执行，请在 App 内逐条确认。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B15"/>
 </worksheet>
 </file>
 
@@ -1323,6 +1335,9 @@
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1376,6 +1391,21 @@
           <t xml:space="preserve">备注</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">配种轮次</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">关联配种记录</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">关联配种导入键</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1428,413 +1458,28 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:J2"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新一轮配种</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">导入键</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">母羊耳号</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">发生日期</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">种公羊耳号</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">冻精编号</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">产羔明细</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">圈舍</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">备注</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">示例-lambing-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">E001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-19</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R001</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L001|母羊|3.4|2026-07-19|是|否;死胎1|未知|2.8|2026-07-19|否|是</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">产羔圈</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">导入键</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">羊只耳号</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">母本耳号</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">父本来源</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">种公羊耳号</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">供体登记号</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">修改原因</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">示例-pedigree-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">E001</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">种公羊</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R001</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">核对产羔本后确认</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">导入键</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">方案名称</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">创建日期</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">步骤</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">示例-program-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">同期发情方案</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-19</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0|放栓;12|撤栓;14|配种</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:D2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">导入键</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">耳号</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">圈舍</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">内容</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">发生日期</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">示例-note-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">观察采食情况</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-19</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">导入键</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">孕检间隔天</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">妊娠周期天</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">断奶日龄</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">提前预警天数</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">每日汇总时间</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">示例-rule-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">45</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">150</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">60</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08:00</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1846,94 +1491,100 @@
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">导入键</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">耳号</t>
+    <col min="10" max="10" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">导入键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">母羊耳号</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">品种</t>
+          <t xml:space="preserve">发生日期</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">性别</t>
+          <t xml:space="preserve">种公羊耳号</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">当前胎次</t>
+          <t xml:space="preserve">冻精编号</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">产羔明细</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">圈舍</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">入场日期</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">出生日期</t>
+          <t xml:space="preserve">备注</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">备注</t>
+          <t xml:space="preserve">关联配种记录</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">关联配种导入键</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例-sheep-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A001</t>
+          <t xml:space="preserve">示例-lambing-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">湖羊</t>
+          <t xml:space="preserve">2026-07-19</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">母羊</t>
+          <t xml:space="preserve">R001</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">育肥一圈</t>
+          <t xml:space="preserve">L001|母羊|3.4|2026-07-19|是|否;死胎1|未知|2.8|2026-07-19|否|是</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-19</t>
+          <t xml:space="preserve">产羔圈</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-02-01</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1941,82 +1592,18 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">导入键</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">耳号</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">体重kg</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">发生日期</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">备注</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">示例-weight-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">35.6</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-19</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">晨间称重</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2036,78 +1623,136 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">耳号</t>
+          <t xml:space="preserve">羊只耳号</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">断奶重kg</t>
+          <t xml:space="preserve">母本耳号</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">转入圈舍</t>
+          <t xml:space="preserve">父本来源</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">发生日期</t>
+          <t xml:space="preserve">种公羊耳号</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">出生日期</t>
+          <t xml:space="preserve">供体登记号</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">备注</t>
+          <t xml:space="preserve">修改原因</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例-wean-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A001</t>
+          <t xml:space="preserve">示例-pedigree-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">22.5</t>
+          <t xml:space="preserve">E001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">育肥二圈</t>
+          <t xml:space="preserve">种公羊</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t xml:space="preserve">R001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">核对产羔本后确认</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">导入键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">方案名称</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">创建日期</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">步骤</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">示例-program-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">同期发情方案</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t xml:space="preserve">2026-07-19</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-01</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0|放栓;12|撤栓;14|配种</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2130,53 +1775,133 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">转入圈舍</t>
+          <t xml:space="preserve">圈舍</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">内容</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">发生日期</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">示例-note-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">观察采食情况</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-19</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">导入键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">孕检间隔天</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">妊娠周期天</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">断奶日龄</t>
+        </is>
+      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">备注</t>
+          <t xml:space="preserve">提前预警天数</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">每日汇总时间</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例-transfer-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A001</t>
+          <t xml:space="preserve">示例-rule-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">45</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">育肥二圈</t>
+          <t xml:space="preserve">150</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-19</t>
+          <t xml:space="preserve">60</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2186,40 +1911,141 @@
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">导入键</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">羊只耳号列表</t>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">导入键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">耳号</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">类型</t>
+          <t xml:space="preserve">品种</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">原因</t>
+          <t xml:space="preserve">性别</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">总售卖金额</t>
+          <t xml:space="preserve">当前胎次</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">圈舍</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入场日期</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出生日期</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">示例-sheep-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">湖羊</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">母羊</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">育肥一圈</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-19</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-01</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">导入键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">耳号</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">体重kg</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">发生日期</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">备注</t>
         </is>
@@ -2228,46 +2054,36 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例-remove-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A001;A002</t>
+          <t xml:space="preserve">示例-weight-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">出售</t>
+          <t xml:space="preserve">35.6</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">正常销售</t>
+          <t xml:space="preserve">2026-07-19</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2400</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-19</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">同一行代表同一批离场</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+          <t xml:space="preserve">晨间称重</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2276,36 +2092,42 @@
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">导入键</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">批次名称</t>
+    <col min="7" max="7" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">导入键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">耳号</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">生产目的</t>
+          <t xml:space="preserve">断奶重kg</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">开始日期</t>
+          <t xml:space="preserve">转入圈舍</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">羊只耳号列表</t>
+          <t xml:space="preserve">发生日期</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">出生日期</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">备注</t>
         </is>
       </c>
@@ -2313,41 +2135,46 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例-batch-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026春羔育肥</t>
+          <t xml:space="preserve">示例-wean-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">育肥</t>
+          <t xml:space="preserve">22.5</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-01</t>
+          <t xml:space="preserve">育肥二圈</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A001;A002</t>
+          <t xml:space="preserve">2026-07-19</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">只允许人工选择</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+          <t xml:space="preserve">2026-03-01</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2365,11 +2192,251 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">耳号</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">转入圈舍</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">发生日期</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">示例-transfer-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">育肥二圈</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-19</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">导入键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">羊只耳号列表</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">类型</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">原因</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">总售卖金额</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">发生日期</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">示例-remove-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A001;A002</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出售</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">正常销售</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2400</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-19</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">同一行代表同一批离场</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">导入键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">批次名称</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">生产目的</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">开始日期</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">羊只耳号列表</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">示例-batch-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026春羔育肥</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">育肥</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-01</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A001;A002</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">只允许人工选择</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">导入键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">批次名称</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">耳号</t>
         </is>
       </c>

</xml_diff>